<commit_message>
presubmission doc and results and scripts modification after R1
</commit_message>
<xml_diff>
--- a/results/Supplementary/Appendix S3. MCMC models details.xlsx
+++ b/results/Supplementary/Appendix S3. MCMC models details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioviedo-my.sharepoint.com/personal/espinosaclara_uniovi_es/Documents/IMIB/Softwares/GitHub/Germination_drivers/results/supplementary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="364" documentId="11_3AC01BE7ED5A0CFFFCDFECC8DB8499C3E9B76F3A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EC272E1-003A-4482-ABEC-EE908B0B4F62}"/>
+  <xr:revisionPtr revIDLastSave="371" documentId="11_3AC01BE7ED5A0CFFFCDFECC8DB8499C3E9B76F3A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC1A59BA-F4DA-45D1-ADD6-9D9322A7263E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="39">
   <si>
     <t>post.mean</t>
   </si>
@@ -147,6 +147,24 @@
   </si>
   <si>
     <t>Results with &gt;50% germination in control conditions</t>
+  </si>
+  <si>
+    <t>Germination cues (sp=16)</t>
+  </si>
+  <si>
+    <t>Water limitation (sp= 16)</t>
+  </si>
+  <si>
+    <t>Control conditions (sp=16)  (Multinomial family)</t>
+  </si>
+  <si>
+    <t>Darkness conditions (sp=16)  (Multinomial family)</t>
+  </si>
+  <si>
+    <t>Constant temperatures conditions (n=16)  (Multinomial family)</t>
+  </si>
+  <si>
+    <t>Water limitation (sp =16) (Exponential family)</t>
   </si>
 </sst>
 </file>
@@ -386,14 +404,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -404,11 +419,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -785,44 +803,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="27"/>
-      <c r="P2" s="27"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
     </row>
     <row r="3" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -830,45 +848,45 @@
       </c>
     </row>
     <row r="4" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="25"/>
-      <c r="J4" s="25"/>
-      <c r="K4" s="25"/>
-      <c r="L4" s="25"/>
-      <c r="M4" s="25"/>
-      <c r="N4" s="25"/>
-      <c r="O4" s="25"/>
-      <c r="P4" s="26"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="25"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="23"/>
-      <c r="H5" s="21" t="s">
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="28"/>
+      <c r="H5" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="23"/>
-      <c r="N5" s="21" t="s">
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="28"/>
+      <c r="N5" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="22"/>
-      <c r="P5" s="23"/>
+      <c r="O5" s="27"/>
+      <c r="P5" s="28"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -1130,45 +1148,45 @@
       <c r="A14" s="1"/>
     </row>
     <row r="15" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="25"/>
-      <c r="J15" s="25"/>
-      <c r="K15" s="25"/>
-      <c r="L15" s="25"/>
-      <c r="M15" s="25"/>
-      <c r="N15" s="25"/>
-      <c r="O15" s="25"/>
-      <c r="P15" s="26"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="24"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="24"/>
+      <c r="L15" s="24"/>
+      <c r="M15" s="24"/>
+      <c r="N15" s="24"/>
+      <c r="O15" s="24"/>
+      <c r="P15" s="25"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="23"/>
-      <c r="H16" s="21" t="s">
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="28"/>
+      <c r="H16" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="I16" s="22"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
-      <c r="L16" s="23"/>
-      <c r="N16" s="21" t="s">
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
+      <c r="K16" s="27"/>
+      <c r="L16" s="28"/>
+      <c r="N16" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="O16" s="22"/>
-      <c r="P16" s="23"/>
+      <c r="O16" s="27"/>
+      <c r="P16" s="28"/>
     </row>
     <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
@@ -1711,49 +1729,49 @@
       </c>
     </row>
     <row r="39" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="24" t="s">
+      <c r="A39" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B39" s="25"/>
-      <c r="C39" s="25"/>
-      <c r="D39" s="25"/>
-      <c r="E39" s="25"/>
-      <c r="F39" s="25"/>
-      <c r="G39" s="25"/>
-      <c r="H39" s="25"/>
-      <c r="I39" s="25"/>
-      <c r="J39" s="25"/>
-      <c r="K39" s="25"/>
-      <c r="L39" s="25"/>
-      <c r="M39" s="25"/>
-      <c r="N39" s="25"/>
-      <c r="O39" s="25"/>
-      <c r="P39" s="26"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="24"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="24"/>
+      <c r="H39" s="24"/>
+      <c r="I39" s="24"/>
+      <c r="J39" s="24"/>
+      <c r="K39" s="24"/>
+      <c r="L39" s="24"/>
+      <c r="M39" s="24"/>
+      <c r="N39" s="24"/>
+      <c r="O39" s="24"/>
+      <c r="P39" s="25"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B40" s="21" t="s">
+      <c r="B40" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C40" s="22"/>
-      <c r="D40" s="22"/>
-      <c r="E40" s="22"/>
-      <c r="F40" s="23"/>
-      <c r="H40" s="21" t="s">
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="28"/>
+      <c r="H40" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="I40" s="22"/>
-      <c r="J40" s="22"/>
-      <c r="K40" s="22"/>
-      <c r="L40" s="23"/>
-      <c r="N40" s="21" t="s">
+      <c r="I40" s="27"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="27"/>
+      <c r="L40" s="28"/>
+      <c r="N40" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="O40" s="22"/>
-      <c r="P40" s="23"/>
+      <c r="O40" s="27"/>
+      <c r="P40" s="28"/>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="B41" s="20" t="s">
         <v>0</v>
@@ -1914,7 +1932,7 @@
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B46" s="4"/>
       <c r="F46" s="5"/>
@@ -2011,45 +2029,45 @@
       <c r="A49" s="1"/>
     </row>
     <row r="50" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="24" t="s">
+      <c r="A50" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="25"/>
-      <c r="C50" s="25"/>
-      <c r="D50" s="25"/>
-      <c r="E50" s="25"/>
-      <c r="F50" s="25"/>
-      <c r="G50" s="25"/>
-      <c r="H50" s="25"/>
-      <c r="I50" s="25"/>
-      <c r="J50" s="25"/>
-      <c r="K50" s="25"/>
-      <c r="L50" s="25"/>
-      <c r="M50" s="25"/>
-      <c r="N50" s="25"/>
-      <c r="O50" s="25"/>
-      <c r="P50" s="26"/>
+      <c r="B50" s="24"/>
+      <c r="C50" s="24"/>
+      <c r="D50" s="24"/>
+      <c r="E50" s="24"/>
+      <c r="F50" s="24"/>
+      <c r="G50" s="24"/>
+      <c r="H50" s="24"/>
+      <c r="I50" s="24"/>
+      <c r="J50" s="24"/>
+      <c r="K50" s="24"/>
+      <c r="L50" s="24"/>
+      <c r="M50" s="24"/>
+      <c r="N50" s="24"/>
+      <c r="O50" s="24"/>
+      <c r="P50" s="25"/>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B51" s="21" t="s">
+      <c r="B51" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C51" s="22"/>
-      <c r="D51" s="22"/>
-      <c r="E51" s="22"/>
-      <c r="F51" s="23"/>
-      <c r="H51" s="21" t="s">
+      <c r="C51" s="27"/>
+      <c r="D51" s="27"/>
+      <c r="E51" s="27"/>
+      <c r="F51" s="28"/>
+      <c r="H51" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="I51" s="22"/>
-      <c r="J51" s="22"/>
-      <c r="K51" s="22"/>
-      <c r="L51" s="23"/>
-      <c r="N51" s="21" t="s">
+      <c r="I51" s="27"/>
+      <c r="J51" s="27"/>
+      <c r="K51" s="27"/>
+      <c r="L51" s="28"/>
+      <c r="N51" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="O51" s="22"/>
-      <c r="P51" s="23"/>
+      <c r="O51" s="27"/>
+      <c r="P51" s="28"/>
     </row>
     <row r="52" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
@@ -2187,7 +2205,7 @@
     </row>
     <row r="56" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="12" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B56" s="4"/>
       <c r="F56" s="5"/>
@@ -2290,7 +2308,7 @@
     </row>
     <row r="60" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="13" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="F60" s="5"/>
       <c r="H60" s="4"/>
@@ -2392,7 +2410,7 @@
     </row>
     <row r="64" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="13" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="F64" s="5"/>
       <c r="H64" s="4"/>
@@ -2494,7 +2512,7 @@
     </row>
     <row r="68" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A68" s="13" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="F68" s="5"/>
       <c r="H68" s="4"/>
@@ -2536,8 +2554,15 @@
       <c r="L69" s="5">
         <v>7420</v>
       </c>
-      <c r="N69" s="4"/>
-      <c r="P69" s="5"/>
+      <c r="N69" s="4">
+        <v>0.73</v>
+      </c>
+      <c r="O69">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="P69" s="5">
+        <v>0.96</v>
+      </c>
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
@@ -2581,13 +2606,10 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="H16:L16"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="A39:P39"/>
-    <mergeCell ref="B40:F40"/>
     <mergeCell ref="H40:L40"/>
     <mergeCell ref="N40:P40"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
     <mergeCell ref="A50:P50"/>
     <mergeCell ref="B51:F51"/>
     <mergeCell ref="H51:L51"/>
@@ -2597,8 +2619,11 @@
     <mergeCell ref="H5:L5"/>
     <mergeCell ref="N5:P5"/>
     <mergeCell ref="A15:P15"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="H16:L16"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="A39:P39"/>
+    <mergeCell ref="B40:F40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="60" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
post-acceptance figures and supplementary
</commit_message>
<xml_diff>
--- a/results/Supplementary/Appendix S3. MCMC models details.xlsx
+++ b/results/Supplementary/Appendix S3. MCMC models details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioviedo-my.sharepoint.com/personal/espinosaclara_uniovi_es/Documents/IMIB/Softwares/GitHub/Germination_drivers/results/supplementary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="371" documentId="11_3AC01BE7ED5A0CFFFCDFECC8DB8499C3E9B76F3A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC1A59BA-F4DA-45D1-ADD6-9D9322A7263E}"/>
+  <xr:revisionPtr revIDLastSave="374" documentId="11_3AC01BE7ED5A0CFFFCDFECC8DB8499C3E9B76F3A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A209831-CE08-451F-894E-5E3DE7B1878B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-18855" yWindow="345" windowWidth="14175" windowHeight="14745" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
@@ -96,11 +96,50 @@
     <t>Habitat Temperate</t>
   </si>
   <si>
-    <t>Appendix S3. MCMC germination model results</t>
+    <t>Germination cues (sp=30)</t>
+  </si>
+  <si>
+    <t>Water limitation (sp= 30)</t>
+  </si>
+  <si>
+    <t>Control conditions (sp=30)  (Multinomial family)</t>
+  </si>
+  <si>
+    <t>Darkness conditions (sp=30)  (Multinomial family)</t>
+  </si>
+  <si>
+    <t>Constant temperatures conditions (n=30)  (Multinomial family)</t>
+  </si>
+  <si>
+    <t>Water limitation (sp =30) (Exponential family)</t>
+  </si>
+  <si>
+    <t>Results with &gt;10% germination in control conditions</t>
+  </si>
+  <si>
+    <t>Results with &gt;50% germination in control conditions</t>
+  </si>
+  <si>
+    <t>Germination cues (sp=16)</t>
+  </si>
+  <si>
+    <t>Water limitation (sp= 16)</t>
+  </si>
+  <si>
+    <t>Control conditions (sp=16)  (Multinomial family)</t>
+  </si>
+  <si>
+    <t>Darkness conditions (sp=16)  (Multinomial family)</t>
+  </si>
+  <si>
+    <t>Constant temperatures conditions (n=16)  (Multinomial family)</t>
+  </si>
+  <si>
+    <t>Water limitation (sp =16) (Exponential family)</t>
   </si>
   <si>
     <r>
-      <t>The Alpine Germination Syndrome differs between Temperate and Mediterranean habitats.</t>
+      <t xml:space="preserve">Supporting Information to the paper Espinosa del Alba et al., 2026. The Alpine Germination Syndrome differs between Temperate and Mediterranean habitats. </t>
     </r>
     <r>
       <rPr>
@@ -111,7 +150,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> Journal of Vegetation Science</t>
+      <t>Journal of Vegetation Science</t>
     </r>
     <r>
       <rPr>
@@ -125,46 +164,7 @@
     </r>
   </si>
   <si>
-    <t>Germination cues (sp=30)</t>
-  </si>
-  <si>
-    <t>Water limitation (sp= 30)</t>
-  </si>
-  <si>
-    <t>Control conditions (sp=30)  (Multinomial family)</t>
-  </si>
-  <si>
-    <t>Darkness conditions (sp=30)  (Multinomial family)</t>
-  </si>
-  <si>
-    <t>Constant temperatures conditions (n=30)  (Multinomial family)</t>
-  </si>
-  <si>
-    <t>Water limitation (sp =30) (Exponential family)</t>
-  </si>
-  <si>
-    <t>Results with &gt;10% germination in control conditions</t>
-  </si>
-  <si>
-    <t>Results with &gt;50% germination in control conditions</t>
-  </si>
-  <si>
-    <t>Germination cues (sp=16)</t>
-  </si>
-  <si>
-    <t>Water limitation (sp= 16)</t>
-  </si>
-  <si>
-    <t>Control conditions (sp=16)  (Multinomial family)</t>
-  </si>
-  <si>
-    <t>Darkness conditions (sp=16)  (Multinomial family)</t>
-  </si>
-  <si>
-    <t>Constant temperatures conditions (n=16)  (Multinomial family)</t>
-  </si>
-  <si>
-    <t>Water limitation (sp =16) (Exponential family)</t>
+    <t>Appendix S3. MCMC-GLMM germination model results</t>
   </si>
 </sst>
 </file>
@@ -207,18 +207,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="14">
@@ -376,7 +370,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -397,18 +391,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -419,14 +414,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -803,96 +795,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
+      <c r="A1" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
+      <c r="P1" s="25"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="22" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
+      <c r="A2" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
     </row>
     <row r="3" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
-      <c r="J4" s="24"/>
-      <c r="K4" s="24"/>
-      <c r="L4" s="24"/>
-      <c r="M4" s="24"/>
-      <c r="N4" s="24"/>
-      <c r="O4" s="24"/>
-      <c r="P4" s="25"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="24"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="28"/>
-      <c r="H5" s="26" t="s">
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="21"/>
+      <c r="H5" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
-      <c r="K5" s="27"/>
-      <c r="L5" s="28"/>
-      <c r="N5" s="26" t="s">
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="21"/>
+      <c r="N5" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="27"/>
-      <c r="P5" s="28"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="21"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="16" t="s">
         <v>0</v>
       </c>
       <c r="C6" t="s">
@@ -990,7 +982,7 @@
       <c r="E8">
         <v>9000</v>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="5">
         <v>4.44E-4</v>
       </c>
       <c r="H8" s="4" t="s">
@@ -1051,7 +1043,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B11" s="4"/>
       <c r="F11" s="5"/>
@@ -1120,7 +1112,7 @@
       <c r="E13" s="2">
         <v>9000</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="7" t="s">
         <v>11</v>
       </c>
       <c r="G13" s="2"/>
@@ -1148,45 +1140,45 @@
       <c r="A14" s="1"/>
     </row>
     <row r="15" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="23" t="s">
+      <c r="A15" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="24"/>
-      <c r="J15" s="24"/>
-      <c r="K15" s="24"/>
-      <c r="L15" s="24"/>
-      <c r="M15" s="24"/>
-      <c r="N15" s="24"/>
-      <c r="O15" s="24"/>
-      <c r="P15" s="25"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="23"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="23"/>
+      <c r="M15" s="23"/>
+      <c r="N15" s="23"/>
+      <c r="O15" s="23"/>
+      <c r="P15" s="24"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="28"/>
-      <c r="H16" s="26" t="s">
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="21"/>
+      <c r="H16" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
-      <c r="K16" s="27"/>
-      <c r="L16" s="28"/>
-      <c r="N16" s="26" t="s">
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="20"/>
+      <c r="L16" s="21"/>
+      <c r="N16" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="O16" s="27"/>
-      <c r="P16" s="28"/>
+      <c r="O16" s="20"/>
+      <c r="P16" s="21"/>
     </row>
     <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
@@ -1290,7 +1282,7 @@
       <c r="E19" s="2">
         <v>3427</v>
       </c>
-      <c r="F19" s="15">
+      <c r="F19" s="7">
         <v>5.3299999999999997E-3</v>
       </c>
       <c r="G19" s="2"/>
@@ -1324,7 +1316,7 @@
     </row>
     <row r="21" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B21" s="4"/>
       <c r="F21" s="5"/>
@@ -1427,7 +1419,7 @@
     </row>
     <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F25" s="5"/>
       <c r="H25" s="4"/>
@@ -1442,13 +1434,13 @@
       <c r="B26" s="4">
         <v>-0.61460000000000004</v>
       </c>
-      <c r="C26" s="16">
+      <c r="C26" s="14">
         <v>-5.3738999999999999</v>
       </c>
-      <c r="D26" s="16">
+      <c r="D26" s="14">
         <v>3.3336999999999999</v>
       </c>
-      <c r="E26" s="16">
+      <c r="E26" s="14">
         <v>7772</v>
       </c>
       <c r="F26" s="17">
@@ -1486,16 +1478,16 @@
       <c r="B27" s="6">
         <v>-0.31990000000000002</v>
       </c>
-      <c r="C27" s="18">
+      <c r="C27" s="15">
         <v>-1.9148000000000001</v>
       </c>
-      <c r="D27" s="18">
+      <c r="D27" s="15">
         <v>1.1971000000000001</v>
       </c>
-      <c r="E27" s="18">
+      <c r="E27" s="15">
         <v>9007</v>
       </c>
-      <c r="F27" s="19">
+      <c r="F27" s="18">
         <v>0.69199999999999995</v>
       </c>
       <c r="G27" s="2"/>
@@ -1529,7 +1521,7 @@
     </row>
     <row r="29" spans="1:16" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F29" s="5"/>
       <c r="H29" s="4"/>
@@ -1631,7 +1623,7 @@
     </row>
     <row r="33" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F33" s="5"/>
       <c r="H33" s="4"/>
@@ -1646,13 +1638,13 @@
       <c r="B34" s="4">
         <v>-4.0967000000000002</v>
       </c>
-      <c r="C34" s="16">
+      <c r="C34" s="14">
         <v>-4.8537999999999997</v>
       </c>
-      <c r="D34" s="16">
+      <c r="D34" s="14">
         <v>-3.2675000000000001</v>
       </c>
-      <c r="E34" s="16">
+      <c r="E34" s="14">
         <v>8290</v>
       </c>
       <c r="F34" s="17" t="s">
@@ -1690,16 +1682,16 @@
       <c r="B35" s="6">
         <v>-0.38090000000000002</v>
       </c>
-      <c r="C35" s="18">
+      <c r="C35" s="15">
         <v>-0.94369999999999998</v>
       </c>
-      <c r="D35" s="18">
+      <c r="D35" s="15">
         <v>0.223</v>
       </c>
-      <c r="E35" s="18">
+      <c r="E35" s="15">
         <v>6323</v>
       </c>
-      <c r="F35" s="19">
+      <c r="F35" s="18">
         <v>0.18099999999999999</v>
       </c>
       <c r="G35" s="2"/>
@@ -1725,55 +1717,55 @@
     </row>
     <row r="38" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="39" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="23" t="s">
+      <c r="A39" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="B39" s="24"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="24"/>
-      <c r="E39" s="24"/>
-      <c r="F39" s="24"/>
-      <c r="G39" s="24"/>
-      <c r="H39" s="24"/>
-      <c r="I39" s="24"/>
-      <c r="J39" s="24"/>
-      <c r="K39" s="24"/>
-      <c r="L39" s="24"/>
-      <c r="M39" s="24"/>
-      <c r="N39" s="24"/>
-      <c r="O39" s="24"/>
-      <c r="P39" s="25"/>
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="23"/>
+      <c r="F39" s="23"/>
+      <c r="G39" s="23"/>
+      <c r="H39" s="23"/>
+      <c r="I39" s="23"/>
+      <c r="J39" s="23"/>
+      <c r="K39" s="23"/>
+      <c r="L39" s="23"/>
+      <c r="M39" s="23"/>
+      <c r="N39" s="23"/>
+      <c r="O39" s="23"/>
+      <c r="P39" s="24"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B40" s="26" t="s">
+      <c r="B40" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="28"/>
-      <c r="H40" s="26" t="s">
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
+      <c r="F40" s="21"/>
+      <c r="H40" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="I40" s="27"/>
-      <c r="J40" s="27"/>
-      <c r="K40" s="27"/>
-      <c r="L40" s="28"/>
-      <c r="N40" s="26" t="s">
+      <c r="I40" s="20"/>
+      <c r="J40" s="20"/>
+      <c r="K40" s="20"/>
+      <c r="L40" s="21"/>
+      <c r="N40" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="O40" s="27"/>
-      <c r="P40" s="28"/>
+      <c r="O40" s="20"/>
+      <c r="P40" s="21"/>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B41" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B41" s="16" t="s">
         <v>0</v>
       </c>
       <c r="C41" t="s">
@@ -1871,7 +1863,7 @@
       <c r="E43">
         <v>8491</v>
       </c>
-      <c r="F43" s="14">
+      <c r="F43" s="5">
         <v>6.6699999999999995E-4</v>
       </c>
       <c r="H43" s="4" t="s">
@@ -1932,7 +1924,7 @@
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B46" s="4"/>
       <c r="F46" s="5"/>
@@ -2001,7 +1993,7 @@
       <c r="E48" s="2">
         <v>9264</v>
       </c>
-      <c r="F48" s="15" t="s">
+      <c r="F48" s="7" t="s">
         <v>11</v>
       </c>
       <c r="G48" s="2"/>
@@ -2029,45 +2021,45 @@
       <c r="A49" s="1"/>
     </row>
     <row r="50" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="23" t="s">
+      <c r="A50" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="24"/>
-      <c r="C50" s="24"/>
-      <c r="D50" s="24"/>
-      <c r="E50" s="24"/>
-      <c r="F50" s="24"/>
-      <c r="G50" s="24"/>
-      <c r="H50" s="24"/>
-      <c r="I50" s="24"/>
-      <c r="J50" s="24"/>
-      <c r="K50" s="24"/>
-      <c r="L50" s="24"/>
-      <c r="M50" s="24"/>
-      <c r="N50" s="24"/>
-      <c r="O50" s="24"/>
-      <c r="P50" s="25"/>
+      <c r="B50" s="23"/>
+      <c r="C50" s="23"/>
+      <c r="D50" s="23"/>
+      <c r="E50" s="23"/>
+      <c r="F50" s="23"/>
+      <c r="G50" s="23"/>
+      <c r="H50" s="23"/>
+      <c r="I50" s="23"/>
+      <c r="J50" s="23"/>
+      <c r="K50" s="23"/>
+      <c r="L50" s="23"/>
+      <c r="M50" s="23"/>
+      <c r="N50" s="23"/>
+      <c r="O50" s="23"/>
+      <c r="P50" s="24"/>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B51" s="26" t="s">
+      <c r="B51" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C51" s="27"/>
-      <c r="D51" s="27"/>
-      <c r="E51" s="27"/>
-      <c r="F51" s="28"/>
-      <c r="H51" s="26" t="s">
+      <c r="C51" s="20"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="20"/>
+      <c r="F51" s="21"/>
+      <c r="H51" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="I51" s="27"/>
-      <c r="J51" s="27"/>
-      <c r="K51" s="27"/>
-      <c r="L51" s="28"/>
-      <c r="N51" s="26" t="s">
+      <c r="I51" s="20"/>
+      <c r="J51" s="20"/>
+      <c r="K51" s="20"/>
+      <c r="L51" s="21"/>
+      <c r="N51" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="O51" s="27"/>
-      <c r="P51" s="28"/>
+      <c r="O51" s="20"/>
+      <c r="P51" s="21"/>
     </row>
     <row r="52" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
@@ -2171,7 +2163,7 @@
       <c r="E54" s="2">
         <v>3427</v>
       </c>
-      <c r="F54" s="15">
+      <c r="F54" s="7">
         <v>5.3299999999999997E-3</v>
       </c>
       <c r="G54" s="2"/>
@@ -2205,7 +2197,7 @@
     </row>
     <row r="56" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B56" s="4"/>
       <c r="F56" s="5"/>
@@ -2308,7 +2300,7 @@
     </row>
     <row r="60" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="13" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F60" s="5"/>
       <c r="H60" s="4"/>
@@ -2410,7 +2402,7 @@
     </row>
     <row r="64" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F64" s="5"/>
       <c r="H64" s="4"/>
@@ -2512,7 +2504,7 @@
     </row>
     <row r="68" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A68" s="13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F68" s="5"/>
       <c r="H68" s="4"/>
@@ -2606,8 +2598,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="H40:L40"/>
-    <mergeCell ref="N40:P40"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:P2"/>
     <mergeCell ref="A50:P50"/>
@@ -2624,6 +2614,8 @@
     <mergeCell ref="N16:P16"/>
     <mergeCell ref="A39:P39"/>
     <mergeCell ref="B40:F40"/>
+    <mergeCell ref="H40:L40"/>
+    <mergeCell ref="N40:P40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="60" orientation="portrait" r:id="rId1"/>

</xml_diff>